<commit_message>
Updated Scenarios and Solver settings
</commit_message>
<xml_diff>
--- a/data/2.b_Hybrider_Netzzugang_2025_3%/Power_Parameters.xlsx
+++ b/data/2.b_Hybrider_Netzzugang_2025_3%/Power_Parameters.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\LEGO-Pyomo\data\2.b_Hybrider_Netzzugang_2025_3%\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\LEGO-Pyomo\data\2.b_Hybrider_Netzzugang_2035_5%\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4390B8A4-A351-4F35-AB08-70ACFE203E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDED682B-B4F5-4A6F-97AF-59C5209C152F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="910" yWindow="5070" windowWidth="28800" windowHeight="15450" tabRatio="958" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="958" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Power Parameters" sheetId="121" r:id="rId1"/>
@@ -1491,7 +1491,7 @@
         <v>82</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F32" s="1" t="s">
         <v>83</v>
@@ -2160,15 +2160,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101004934E3CB1C58BA43BC6E229E2BF20201" ma:contentTypeVersion="4" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="e33ccc94e63df24f58cb47229b46e190">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87003a75-b64f-4b22-bf19-aa30740e3d46" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0f0f7a5bb162b669de9ce8ff8278c29f" ns2:_="">
     <xsd:import namespace="87003a75-b64f-4b22-bf19-aa30740e3d46"/>
@@ -2314,6 +2305,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0155F7A0-74CD-4575-8C0B-A34C113F80FE}">
   <ds:schemaRefs>
@@ -2331,14 +2331,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13778B2C-CE05-4B32-8196-2F381FEAC95A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{773946F7-566C-458F-95C9-79B0CCE20E87}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2354,4 +2346,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13778B2C-CE05-4B32-8196-2F381FEAC95A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>